<commit_message>
Replace placeholder module bucket
Replace the generic Others bucket with real module menu items for store management, repair and maintenance, salvage, budget planning, inspectorate, administration, communication, and DMS. Keep the sidebar hierarchy aligned in the navigation defaults and localized reference templates.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Services/Iam/src/Iam.Api/ReferenceData/Navigation/us_military_module_navigation_template_ar.xlsx
+++ b/Services/Iam/src/Iam.Api/ReferenceData/Navigation/us_military_module_navigation_template_ar.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,17 +564,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>store-management</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>store-management</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>????</t>
+          <t>????? ???????</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -582,10 +582,206 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>apps</t>
+          <t>inventory_2</t>
         </is>
       </c>
       <c r="F6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>repair-maintenance</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>repair-maintenance</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>??????? ????????</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>60</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>salvage</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>salvage</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>???????</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>recycling</t>
+        </is>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>budget-planning</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>budget-planning</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>????????? ????????</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>account_balance_wallet</t>
+        </is>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>inspectorate</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>inspectorate</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>?????? ?????????</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>manage_search</t>
+        </is>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>???????</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>admin_panel_settings</t>
+        </is>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>?????????</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>110</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dms</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>dms</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>????? ?????????</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>120</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -600,7 +796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1973,18 +2169,18 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>store-management</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>store-management</t>
+          <t>stock-levels</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>????? ??????</t>
+          <t>??????? ???????</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -1992,7 +2188,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>inventory_2</t>
+          <t>stacked_bar_chart</t>
         </is>
       </c>
       <c r="G44" t="b">
@@ -2002,30 +2198,26 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>store-management</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>stock-levels</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>store-management</t>
-        </is>
-      </c>
+          <t>reorder-alerts</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>??????? ???????</t>
+          <t>??????? ????? ?????</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>stacked_bar_chart</t>
+          <t>notification_important</t>
         </is>
       </c>
       <c r="G45" t="b">
@@ -2035,30 +2227,26 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>store-management</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>reorder-alerts</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>store-management</t>
-        </is>
-      </c>
+          <t>asset-cards</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>??????? ????? ?????</t>
+          <t>?????? ??????</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>notification_important</t>
+          <t>badge</t>
         </is>
       </c>
       <c r="G46" t="b">
@@ -2068,30 +2256,26 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>repair-maintenance</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>asset-cards</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>store-management</t>
-        </is>
-      </c>
+          <t>work-orders</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>?????? ??????</t>
+          <t>????? ?????</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>badge</t>
+          <t>handyman</t>
         </is>
       </c>
       <c r="G47" t="b">
@@ -2101,18 +2285,18 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>repair-maintenance</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>repair-maintenance</t>
+          <t>maintenance-schedule</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>??????? ????????</t>
+          <t>???? ???????</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -2120,7 +2304,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>calendar_month</t>
         </is>
       </c>
       <c r="G48" t="b">
@@ -2130,30 +2314,26 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>repair-maintenance</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>work-orders</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>repair-maintenance</t>
-        </is>
-      </c>
+          <t>parts-usage</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>????? ?????</t>
+          <t>??????? ?????</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>handyman</t>
+          <t>precision_manufacturing</t>
         </is>
       </c>
       <c r="G49" t="b">
@@ -2163,30 +2343,26 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>salvage</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>maintenance-schedule</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>repair-maintenance</t>
-        </is>
-      </c>
+          <t>recovery-cases</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>???? ???????</t>
+          <t>????? ?????????</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>calendar_month</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="G50" t="b">
@@ -2196,30 +2372,26 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>salvage</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>parts-usage</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>repair-maintenance</t>
-        </is>
-      </c>
+          <t>disposal-records</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>??????? ?????</t>
+          <t>????? ???????</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>precision_manufacturing</t>
+          <t>delete_forever</t>
         </is>
       </c>
       <c r="G51" t="b">
@@ -2229,26 +2401,26 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>budget-planning</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>salvage</t>
+          <t>allocations</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>???????</t>
+          <t>?????????</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>recycling</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="G52" t="b">
@@ -2258,30 +2430,26 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>budget-planning</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>recovery-cases</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>salvage</t>
-        </is>
-      </c>
+          <t>spend-forecast</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>????? ?????????</t>
+          <t>???? ???????</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>trending_up</t>
         </is>
       </c>
       <c r="G53" t="b">
@@ -2291,30 +2459,26 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>budget-planning</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>disposal-records</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>salvage</t>
-        </is>
-      </c>
+          <t>budget-vs-actual</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>????? ???????</t>
+          <t>????????? ????? ??????</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>delete_forever</t>
+          <t>compare_arrows</t>
         </is>
       </c>
       <c r="G54" t="b">
@@ -2324,26 +2488,26 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>inspectorate</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>budget-planning</t>
+          <t>audits</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>????????? ????????</t>
+          <t>?????????</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>account_balance_wallet</t>
+          <t>search_check</t>
         </is>
       </c>
       <c r="G55" t="b">
@@ -2353,30 +2517,26 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>inspectorate</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>allocations</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>budget-planning</t>
-        </is>
-      </c>
+          <t>findings</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>?????????</t>
+          <t>???????</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>rule_folder</t>
         </is>
       </c>
       <c r="G56" t="b">
@@ -2386,30 +2546,26 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>inspectorate</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>spend-forecast</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>budget-planning</t>
-        </is>
-      </c>
+          <t>corrective-actions</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>???? ???????</t>
+          <t>????????? ?????????</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>trending_up</t>
+          <t>fact_check</t>
         </is>
       </c>
       <c r="G57" t="b">
@@ -2419,30 +2575,26 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>budget-vs-actual</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>budget-planning</t>
-        </is>
-      </c>
+          <t>departments</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>????????? ????? ??????</t>
+          <t>???????</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>compare_arrows</t>
+          <t>corporate_fare</t>
         </is>
       </c>
       <c r="G58" t="b">
@@ -2452,26 +2604,26 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>inspectorate</t>
+          <t>roles</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>?????? ?????????</t>
+          <t>???????</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>manage_search</t>
+          <t>admin_panel_settings</t>
         </is>
       </c>
       <c r="G59" t="b">
@@ -2481,30 +2633,26 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>audits</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>inspectorate</t>
-        </is>
-      </c>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>?????????</t>
+          <t>??????????</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>search_check</t>
+          <t>groups</t>
         </is>
       </c>
       <c r="G60" t="b">
@@ -2514,30 +2662,26 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>communication</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>findings</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>inspectorate</t>
-        </is>
-      </c>
+          <t>channels</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>???????</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>rule_folder</t>
+          <t>forum</t>
         </is>
       </c>
       <c r="G61" t="b">
@@ -2547,30 +2691,26 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>communication</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>corrective-actions</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>inspectorate</t>
-        </is>
-      </c>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>????????? ?????????</t>
+          <t>?????????</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>fact_check</t>
+          <t>campaign</t>
         </is>
       </c>
       <c r="G62" t="b">
@@ -2580,12 +2720,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>communication</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>messages</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -2595,11 +2735,11 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>admin_panel_settings</t>
+          <t>message</t>
         </is>
       </c>
       <c r="G63" t="b">
@@ -2609,22 +2749,18 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>dms</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>departments</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>administration</t>
-        </is>
-      </c>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>???????</t>
+          <t>?????????</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -2632,7 +2768,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>corporate_fare</t>
+          <t>description</t>
         </is>
       </c>
       <c r="G64" t="b">
@@ -2642,22 +2778,18 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>dms</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>roles</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>administration</t>
-        </is>
-      </c>
+          <t>folders</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>???????</t>
+          <t>????????</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -2665,7 +2797,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>admin_panel_settings</t>
+          <t>folder</t>
         </is>
       </c>
       <c r="G65" t="b">
@@ -2675,22 +2807,18 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>dms</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>users</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>administration</t>
-        </is>
-      </c>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>??????????</t>
+          <t>?????????</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -2698,266 +2826,10 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>groups</t>
+          <t>history</t>
         </is>
       </c>
       <c r="G66" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>communication</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>?????????</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>70</v>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>chat</t>
-        </is>
-      </c>
-      <c r="G67" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>channels</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>communication</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>???????</t>
-        </is>
-      </c>
-      <c r="E68" t="n">
-        <v>10</v>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>forum</t>
-        </is>
-      </c>
-      <c r="G68" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>announcements</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>communication</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>?????????</t>
-        </is>
-      </c>
-      <c r="E69" t="n">
-        <v>20</v>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>campaign</t>
-        </is>
-      </c>
-      <c r="G69" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>messages</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>communication</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>???????</t>
-        </is>
-      </c>
-      <c r="E70" t="n">
-        <v>30</v>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>message</t>
-        </is>
-      </c>
-      <c r="G70" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>dms</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>????? ?????????</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
-        <v>80</v>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G71" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>documents</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>dms</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>?????????</t>
-        </is>
-      </c>
-      <c r="E72" t="n">
-        <v>10</v>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G72" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>folders</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>dms</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>20</v>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>folder</t>
-        </is>
-      </c>
-      <c r="G73" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>others</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>versions</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>dms</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>?????????</t>
-        </is>
-      </c>
-      <c r="E74" t="n">
-        <v>30</v>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>history</t>
-        </is>
-      </c>
-      <c r="G74" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>